<commit_message>
Generate clinical data summary
</commit_message>
<xml_diff>
--- a/data/metadata_for_eytan-BIDMC_PCBN_UM.xlsx
+++ b/data/metadata_for_eytan-BIDMC_PCBN_UM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adamsowalsky/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://somumaryland-my.sharepoint.com/personal/binbin_wang_som_umaryland_edu/Documents/nih_backup/projects/adam/BBS_Prostate_cancer/BSS_Prostate_cancer/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0F05AE6B-C36D-EA43-A0ED-AFDB1E7511B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{0F05AE6B-C36D-EA43-A0ED-AFDB1E7511B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70573CA3-E550-2945-B85E-712C63B7632F}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="740" windowWidth="24000" windowHeight="17160" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20020" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="2" r:id="rId1"/>
@@ -11758,6 +11758,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:AH712"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
@@ -13066,7 +13067,7 @@
         <v>61.533333333333331</v>
       </c>
     </row>
-    <row r="24" spans="1:18">
+    <row r="24" spans="1:18" hidden="1">
       <c r="A24" s="7" t="s">
         <v>49</v>
       </c>
@@ -13234,7 +13235,7 @@
         <v>65.933333333333337</v>
       </c>
     </row>
-    <row r="27" spans="1:18">
+    <row r="27" spans="1:18" hidden="1">
       <c r="A27" s="7" t="s">
         <v>54</v>
       </c>
@@ -14298,7 +14299,7 @@
         <v>27.733333333333334</v>
       </c>
     </row>
-    <row r="46" spans="1:18">
+    <row r="46" spans="1:18" hidden="1">
       <c r="A46" s="7" t="s">
         <v>82</v>
       </c>
@@ -14466,7 +14467,7 @@
         <v>13.166666666666666</v>
       </c>
     </row>
-    <row r="49" spans="1:18">
+    <row r="49" spans="1:18" hidden="1">
       <c r="A49" s="7" t="s">
         <v>86</v>
       </c>
@@ -14634,7 +14635,7 @@
         <v>29.8</v>
       </c>
     </row>
-    <row r="52" spans="1:18">
+    <row r="52" spans="1:18" hidden="1">
       <c r="A52" s="7" t="s">
         <v>90</v>
       </c>
@@ -14914,7 +14915,7 @@
         <v>25.866666666666667</v>
       </c>
     </row>
-    <row r="57" spans="1:18">
+    <row r="57" spans="1:18" hidden="1">
       <c r="A57" s="7" t="s">
         <v>97</v>
       </c>
@@ -15082,7 +15083,7 @@
         <v>15.366666666666667</v>
       </c>
     </row>
-    <row r="60" spans="1:18">
+    <row r="60" spans="1:18" hidden="1">
       <c r="A60" s="7" t="s">
         <v>101</v>
       </c>
@@ -15362,7 +15363,7 @@
         <v>54.56666666666667</v>
       </c>
     </row>
-    <row r="65" spans="1:18">
+    <row r="65" spans="1:18" hidden="1">
       <c r="A65" s="7" t="s">
         <v>108</v>
       </c>
@@ -15530,7 +15531,7 @@
         <v>12.933333333333334</v>
       </c>
     </row>
-    <row r="68" spans="1:18">
+    <row r="68" spans="1:18" hidden="1">
       <c r="A68" s="7" t="s">
         <v>112</v>
       </c>
@@ -15698,7 +15699,7 @@
         <v>18.033333333333335</v>
       </c>
     </row>
-    <row r="71" spans="1:18">
+    <row r="71" spans="1:18" hidden="1">
       <c r="A71" s="7" t="s">
         <v>116</v>
       </c>
@@ -15866,7 +15867,7 @@
         <v>32.43333333333333</v>
       </c>
     </row>
-    <row r="74" spans="1:18">
+    <row r="74" spans="1:18" hidden="1">
       <c r="A74" s="7" t="s">
         <v>120</v>
       </c>
@@ -16034,7 +16035,7 @@
         <v>39.56666666666667</v>
       </c>
     </row>
-    <row r="77" spans="1:18">
+    <row r="77" spans="1:18" hidden="1">
       <c r="A77" s="7" t="s">
         <v>124</v>
       </c>
@@ -16202,7 +16203,7 @@
         <v>38.43333333333333</v>
       </c>
     </row>
-    <row r="80" spans="1:18">
+    <row r="80" spans="1:18" hidden="1">
       <c r="A80" s="7" t="s">
         <v>128</v>
       </c>
@@ -16482,7 +16483,7 @@
         <v>47.06666666666667</v>
       </c>
     </row>
-    <row r="85" spans="1:18">
+    <row r="85" spans="1:18" hidden="1">
       <c r="A85" s="7" t="s">
         <v>135</v>
       </c>
@@ -16650,7 +16651,7 @@
         <v>48.9</v>
       </c>
     </row>
-    <row r="88" spans="1:18">
+    <row r="88" spans="1:18" hidden="1">
       <c r="A88" s="7" t="s">
         <v>139</v>
       </c>
@@ -16930,7 +16931,7 @@
         <v>51.4</v>
       </c>
     </row>
-    <row r="93" spans="1:18">
+    <row r="93" spans="1:18" hidden="1">
       <c r="A93" s="7" t="s">
         <v>146</v>
       </c>
@@ -17210,7 +17211,7 @@
         <v>63.466666666666669</v>
       </c>
     </row>
-    <row r="98" spans="1:18">
+    <row r="98" spans="1:18" hidden="1">
       <c r="A98" s="7" t="s">
         <v>153</v>
       </c>
@@ -17378,7 +17379,7 @@
         <v>30.966666666666665</v>
       </c>
     </row>
-    <row r="101" spans="1:18">
+    <row r="101" spans="1:18" hidden="1">
       <c r="A101" s="7" t="s">
         <v>157</v>
       </c>
@@ -17658,7 +17659,7 @@
         <v>61.966666666666669</v>
       </c>
     </row>
-    <row r="106" spans="1:18">
+    <row r="106" spans="1:18" hidden="1">
       <c r="A106" s="7" t="s">
         <v>164</v>
       </c>
@@ -17826,7 +17827,7 @@
         <v>42.766666666666666</v>
       </c>
     </row>
-    <row r="109" spans="1:18">
+    <row r="109" spans="1:18" hidden="1">
       <c r="A109" s="7" t="s">
         <v>168</v>
       </c>
@@ -17994,7 +17995,7 @@
         <v>26.466666666666665</v>
       </c>
     </row>
-    <row r="112" spans="1:18">
+    <row r="112" spans="1:18" hidden="1">
       <c r="A112" s="7" t="s">
         <v>172</v>
       </c>
@@ -18162,7 +18163,7 @@
         <v>60.7</v>
       </c>
     </row>
-    <row r="115" spans="1:18">
+    <row r="115" spans="1:18" hidden="1">
       <c r="A115" s="7" t="s">
         <v>176</v>
       </c>
@@ -18442,7 +18443,7 @@
         <v>25.4</v>
       </c>
     </row>
-    <row r="120" spans="1:18">
+    <row r="120" spans="1:18" hidden="1">
       <c r="A120" s="7" t="s">
         <v>183</v>
       </c>
@@ -18610,7 +18611,7 @@
         <v>34.799999999999997</v>
       </c>
     </row>
-    <row r="123" spans="1:18">
+    <row r="123" spans="1:18" hidden="1">
       <c r="A123" s="7" t="s">
         <v>187</v>
       </c>
@@ -18778,7 +18779,7 @@
         <v>49.93333333333333</v>
       </c>
     </row>
-    <row r="126" spans="1:18">
+    <row r="126" spans="1:18" hidden="1">
       <c r="A126" s="7" t="s">
         <v>191</v>
       </c>
@@ -18946,7 +18947,7 @@
         <v>24.366666666666667</v>
       </c>
     </row>
-    <row r="129" spans="1:34">
+    <row r="129" spans="1:34" hidden="1">
       <c r="A129" s="7" t="s">
         <v>195</v>
       </c>
@@ -19144,7 +19145,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="132" spans="1:34">
+    <row r="132" spans="1:34" hidden="1">
       <c r="A132" s="7" t="s">
         <v>199</v>
       </c>
@@ -19312,7 +19313,7 @@
         <v>27.966666666666665</v>
       </c>
     </row>
-    <row r="135" spans="1:34">
+    <row r="135" spans="1:34" hidden="1">
       <c r="A135" s="7" t="s">
         <v>203</v>
       </c>
@@ -19480,7 +19481,7 @@
         <v>36.366666666666667</v>
       </c>
     </row>
-    <row r="138" spans="1:34">
+    <row r="138" spans="1:34" hidden="1">
       <c r="A138" s="7" t="s">
         <v>207</v>
       </c>
@@ -19648,7 +19649,7 @@
         <v>44.266666666666666</v>
       </c>
     </row>
-    <row r="141" spans="1:34">
+    <row r="141" spans="1:34" hidden="1">
       <c r="A141" s="7" t="s">
         <v>211</v>
       </c>
@@ -19816,7 +19817,7 @@
         <v>23.966666666666665</v>
       </c>
     </row>
-    <row r="144" spans="1:34">
+    <row r="144" spans="1:34" hidden="1">
       <c r="A144" s="7" t="s">
         <v>215</v>
       </c>
@@ -19984,7 +19985,7 @@
         <v>36.200000000000003</v>
       </c>
     </row>
-    <row r="147" spans="1:18">
+    <row r="147" spans="1:18" hidden="1">
       <c r="A147" s="7" t="s">
         <v>219</v>
       </c>
@@ -20152,7 +20153,7 @@
         <v>3.6333333333333333</v>
       </c>
     </row>
-    <row r="150" spans="1:18">
+    <row r="150" spans="1:18" hidden="1">
       <c r="A150" s="7" t="s">
         <v>223</v>
       </c>
@@ -20320,7 +20321,7 @@
         <v>12.6</v>
       </c>
     </row>
-    <row r="153" spans="1:18">
+    <row r="153" spans="1:18" hidden="1">
       <c r="A153" s="7" t="s">
         <v>227</v>
       </c>
@@ -20488,7 +20489,7 @@
         <v>12.566666666666666</v>
       </c>
     </row>
-    <row r="156" spans="1:18">
+    <row r="156" spans="1:18" hidden="1">
       <c r="A156" s="7" t="s">
         <v>231</v>
       </c>
@@ -20656,7 +20657,7 @@
         <v>55.033333333333331</v>
       </c>
     </row>
-    <row r="159" spans="1:18">
+    <row r="159" spans="1:18" hidden="1">
       <c r="A159" s="7" t="s">
         <v>235</v>
       </c>
@@ -20824,7 +20825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:18">
+    <row r="162" spans="1:18" hidden="1">
       <c r="A162" s="7" t="s">
         <v>239</v>
       </c>
@@ -20992,7 +20993,7 @@
         <v>6.9</v>
       </c>
     </row>
-    <row r="165" spans="1:18">
+    <row r="165" spans="1:18" hidden="1">
       <c r="A165" s="7" t="s">
         <v>243</v>
       </c>
@@ -21160,7 +21161,7 @@
         <v>23.8</v>
       </c>
     </row>
-    <row r="168" spans="1:18">
+    <row r="168" spans="1:18" hidden="1">
       <c r="A168" s="7" t="s">
         <v>247</v>
       </c>
@@ -21328,7 +21329,7 @@
         <v>12.4</v>
       </c>
     </row>
-    <row r="171" spans="1:18">
+    <row r="171" spans="1:18" hidden="1">
       <c r="A171" s="7" t="s">
         <v>251</v>
       </c>
@@ -21496,7 +21497,7 @@
         <v>14.333333333333334</v>
       </c>
     </row>
-    <row r="174" spans="1:18">
+    <row r="174" spans="1:18" hidden="1">
       <c r="A174" s="7" t="s">
         <v>255</v>
       </c>
@@ -21664,7 +21665,7 @@
         <v>27.166666666666668</v>
       </c>
     </row>
-    <row r="177" spans="1:18">
+    <row r="177" spans="1:18" hidden="1">
       <c r="A177" s="7" t="s">
         <v>259</v>
       </c>
@@ -21832,7 +21833,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="180" spans="1:18">
+    <row r="180" spans="1:18" hidden="1">
       <c r="A180" s="7" t="s">
         <v>263</v>
       </c>
@@ -22000,7 +22001,7 @@
         <v>29.233333333333334</v>
       </c>
     </row>
-    <row r="183" spans="1:18">
+    <row r="183" spans="1:18" hidden="1">
       <c r="A183" s="7" t="s">
         <v>267</v>
       </c>
@@ -22168,7 +22169,7 @@
         <v>26.933333333333334</v>
       </c>
     </row>
-    <row r="186" spans="1:18">
+    <row r="186" spans="1:18" hidden="1">
       <c r="A186" s="7" t="s">
         <v>271</v>
       </c>
@@ -22336,7 +22337,7 @@
         <v>34.633333333333333</v>
       </c>
     </row>
-    <row r="189" spans="1:18">
+    <row r="189" spans="1:18" hidden="1">
       <c r="A189" s="7" t="s">
         <v>275</v>
       </c>
@@ -22504,7 +22505,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="192" spans="1:18">
+    <row r="192" spans="1:18" hidden="1">
       <c r="A192" s="7" t="s">
         <v>279</v>
       </c>
@@ -22672,7 +22673,7 @@
         <v>24.3</v>
       </c>
     </row>
-    <row r="195" spans="1:18">
+    <row r="195" spans="1:18" hidden="1">
       <c r="A195" s="7" t="s">
         <v>283</v>
       </c>
@@ -22840,7 +22841,7 @@
         <v>34.4</v>
       </c>
     </row>
-    <row r="198" spans="1:18">
+    <row r="198" spans="1:18" hidden="1">
       <c r="A198" s="7" t="s">
         <v>287</v>
       </c>
@@ -23008,7 +23009,7 @@
         <v>12.733333333333333</v>
       </c>
     </row>
-    <row r="201" spans="1:18">
+    <row r="201" spans="1:18" hidden="1">
       <c r="A201" s="7" t="s">
         <v>291</v>
       </c>
@@ -23176,7 +23177,7 @@
         <v>26.933333333333334</v>
       </c>
     </row>
-    <row r="204" spans="1:18">
+    <row r="204" spans="1:18" hidden="1">
       <c r="A204" s="7" t="s">
         <v>295</v>
       </c>
@@ -23344,7 +23345,7 @@
         <v>21.1</v>
       </c>
     </row>
-    <row r="207" spans="1:18">
+    <row r="207" spans="1:18" hidden="1">
       <c r="A207" s="7" t="s">
         <v>299</v>
       </c>
@@ -23512,7 +23513,7 @@
         <v>36.200000000000003</v>
       </c>
     </row>
-    <row r="210" spans="1:18">
+    <row r="210" spans="1:18" hidden="1">
       <c r="A210" s="7" t="s">
         <v>303</v>
       </c>
@@ -23680,7 +23681,7 @@
         <v>33.733333333333334</v>
       </c>
     </row>
-    <row r="213" spans="1:18">
+    <row r="213" spans="1:18" hidden="1">
       <c r="A213" s="7" t="s">
         <v>307</v>
       </c>
@@ -23848,7 +23849,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="216" spans="1:18">
+    <row r="216" spans="1:18" hidden="1">
       <c r="A216" s="7" t="s">
         <v>311</v>
       </c>
@@ -24016,7 +24017,7 @@
         <v>12.766666666666667</v>
       </c>
     </row>
-    <row r="219" spans="1:18">
+    <row r="219" spans="1:18" hidden="1">
       <c r="A219" s="7" t="s">
         <v>315</v>
       </c>
@@ -24184,7 +24185,7 @@
         <v>24.8</v>
       </c>
     </row>
-    <row r="222" spans="1:18">
+    <row r="222" spans="1:18" hidden="1">
       <c r="A222" s="7" t="s">
         <v>319</v>
       </c>
@@ -24352,7 +24353,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="225" spans="1:18">
+    <row r="225" spans="1:18" hidden="1">
       <c r="A225" s="7" t="s">
         <v>323</v>
       </c>
@@ -24520,7 +24521,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="228" spans="1:18">
+    <row r="228" spans="1:18" hidden="1">
       <c r="A228" s="2" t="s">
         <v>468</v>
       </c>
@@ -24691,7 +24692,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="231" spans="1:18">
+    <row r="231" spans="1:18" hidden="1">
       <c r="A231" s="2" t="s">
         <v>471</v>
       </c>
@@ -24862,7 +24863,7 @@
         <v>22.368421052631579</v>
       </c>
     </row>
-    <row r="234" spans="1:18">
+    <row r="234" spans="1:18" hidden="1">
       <c r="A234" s="2" t="s">
         <v>474</v>
       </c>
@@ -25033,7 +25034,7 @@
         <v>41.6</v>
       </c>
     </row>
-    <row r="237" spans="1:18">
+    <row r="237" spans="1:18" hidden="1">
       <c r="A237" s="2" t="s">
         <v>477</v>
       </c>
@@ -25204,7 +25205,7 @@
         <v>66.05263157894737</v>
       </c>
     </row>
-    <row r="240" spans="1:18">
+    <row r="240" spans="1:18" hidden="1">
       <c r="A240" s="2" t="s">
         <v>480</v>
       </c>
@@ -25375,7 +25376,7 @@
         <v>32.700000000000003</v>
       </c>
     </row>
-    <row r="243" spans="1:18">
+    <row r="243" spans="1:18" hidden="1">
       <c r="A243" s="2" t="s">
         <v>483</v>
       </c>
@@ -25546,7 +25547,7 @@
         <v>96.019736842105274</v>
       </c>
     </row>
-    <row r="246" spans="1:18">
+    <row r="246" spans="1:18" hidden="1">
       <c r="A246" s="2" t="s">
         <v>486</v>
       </c>
@@ -25717,7 +25718,7 @@
         <v>82.467105263157904</v>
       </c>
     </row>
-    <row r="249" spans="1:18">
+    <row r="249" spans="1:18" hidden="1">
       <c r="A249" s="2" t="s">
         <v>489</v>
       </c>
@@ -25888,7 +25889,7 @@
         <v>98.125</v>
       </c>
     </row>
-    <row r="252" spans="1:18">
+    <row r="252" spans="1:18" hidden="1">
       <c r="A252" s="2" t="s">
         <v>492</v>
       </c>
@@ -26059,7 +26060,7 @@
         <v>54.21052631578948</v>
       </c>
     </row>
-    <row r="255" spans="1:18">
+    <row r="255" spans="1:18" hidden="1">
       <c r="A255" s="2" t="s">
         <v>495</v>
       </c>
@@ -26230,7 +26231,7 @@
         <v>70.099999999999994</v>
       </c>
     </row>
-    <row r="258" spans="1:18">
+    <row r="258" spans="1:18" hidden="1">
       <c r="A258" s="2" t="s">
         <v>498</v>
       </c>
@@ -26401,7 +26402,7 @@
         <v>89.01315789473685</v>
       </c>
     </row>
-    <row r="261" spans="1:18">
+    <row r="261" spans="1:18" hidden="1">
       <c r="A261" s="2" t="s">
         <v>501</v>
       </c>
@@ -26572,7 +26573,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="264" spans="1:18">
+    <row r="264" spans="1:18" hidden="1">
       <c r="A264" s="2" t="s">
         <v>504</v>
       </c>
@@ -26743,7 +26744,7 @@
         <v>93.32236842105263</v>
       </c>
     </row>
-    <row r="267" spans="1:18">
+    <row r="267" spans="1:18" hidden="1">
       <c r="A267" s="2" t="s">
         <v>507</v>
       </c>
@@ -26914,7 +26915,7 @@
         <v>46.5</v>
       </c>
     </row>
-    <row r="270" spans="1:18">
+    <row r="270" spans="1:18" hidden="1">
       <c r="A270" s="2" t="s">
         <v>510</v>
       </c>
@@ -27085,7 +27086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:18">
+    <row r="273" spans="1:18" hidden="1">
       <c r="A273" s="2" t="s">
         <v>513</v>
       </c>
@@ -27256,7 +27257,7 @@
         <v>68.618421052631575</v>
       </c>
     </row>
-    <row r="276" spans="1:18">
+    <row r="276" spans="1:18" hidden="1">
       <c r="A276" s="2" t="s">
         <v>516</v>
       </c>
@@ -27427,7 +27428,7 @@
         <v>46.28289473684211</v>
       </c>
     </row>
-    <row r="279" spans="1:18">
+    <row r="279" spans="1:18" hidden="1">
       <c r="A279" s="2" t="s">
         <v>519</v>
       </c>
@@ -27598,7 +27599,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="282" spans="1:18">
+    <row r="282" spans="1:18" hidden="1">
       <c r="A282" s="2" t="s">
         <v>522</v>
       </c>
@@ -27769,7 +27770,7 @@
         <v>52.9</v>
       </c>
     </row>
-    <row r="285" spans="1:18">
+    <row r="285" spans="1:18" hidden="1">
       <c r="A285" s="2" t="s">
         <v>525</v>
       </c>
@@ -27940,7 +27941,7 @@
         <v>77.861842105263165</v>
       </c>
     </row>
-    <row r="288" spans="1:18">
+    <row r="288" spans="1:18" hidden="1">
       <c r="A288" s="2" t="s">
         <v>528</v>
       </c>
@@ -28111,7 +28112,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="291" spans="1:18">
+    <row r="291" spans="1:18" hidden="1">
       <c r="A291" s="2" t="s">
         <v>531</v>
       </c>
@@ -28282,7 +28283,7 @@
         <v>53.7</v>
       </c>
     </row>
-    <row r="294" spans="1:18">
+    <row r="294" spans="1:18" hidden="1">
       <c r="A294" s="2" t="s">
         <v>534</v>
       </c>
@@ -28453,7 +28454,7 @@
         <v>7.9</v>
       </c>
     </row>
-    <row r="297" spans="1:18">
+    <row r="297" spans="1:18" hidden="1">
       <c r="A297" s="2" t="s">
         <v>537</v>
       </c>
@@ -28624,7 +28625,7 @@
         <v>64.671052631578945</v>
       </c>
     </row>
-    <row r="300" spans="1:18">
+    <row r="300" spans="1:18" hidden="1">
       <c r="A300" s="2" t="s">
         <v>540</v>
       </c>
@@ -28795,7 +28796,7 @@
         <v>12.7</v>
       </c>
     </row>
-    <row r="303" spans="1:18">
+    <row r="303" spans="1:18" hidden="1">
       <c r="A303" s="2" t="s">
         <v>543</v>
       </c>
@@ -28966,7 +28967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="306" spans="1:18">
+    <row r="306" spans="1:18" hidden="1">
       <c r="A306" s="2" t="s">
         <v>546</v>
       </c>
@@ -29137,7 +29138,7 @@
         <v>60.42763157894737</v>
       </c>
     </row>
-    <row r="309" spans="1:18">
+    <row r="309" spans="1:18" hidden="1">
       <c r="A309" s="2" t="s">
         <v>549</v>
       </c>
@@ -29308,7 +29309,7 @@
         <v>74.901315789473685</v>
       </c>
     </row>
-    <row r="312" spans="1:18">
+    <row r="312" spans="1:18" hidden="1">
       <c r="A312" s="2" t="s">
         <v>552</v>
       </c>
@@ -29479,7 +29480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="315" spans="1:18">
+    <row r="315" spans="1:18" hidden="1">
       <c r="A315" s="2" t="s">
         <v>555</v>
       </c>
@@ -29650,7 +29651,7 @@
         <v>62.763157894736842</v>
       </c>
     </row>
-    <row r="318" spans="1:18">
+    <row r="318" spans="1:18" hidden="1">
       <c r="A318" s="2" t="s">
         <v>558</v>
       </c>
@@ -29821,7 +29822,7 @@
         <v>66.51315789473685</v>
       </c>
     </row>
-    <row r="321" spans="1:18">
+    <row r="321" spans="1:18" hidden="1">
       <c r="A321" s="2" t="s">
         <v>561</v>
       </c>
@@ -29992,7 +29993,7 @@
         <v>66.184210526315795</v>
       </c>
     </row>
-    <row r="324" spans="1:18">
+    <row r="324" spans="1:18" hidden="1">
       <c r="A324" s="2" t="s">
         <v>564</v>
       </c>
@@ -30163,7 +30164,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="327" spans="1:18">
+    <row r="327" spans="1:18" hidden="1">
       <c r="A327" s="2" t="s">
         <v>567</v>
       </c>
@@ -30334,7 +30335,7 @@
         <v>57.828947368421055</v>
       </c>
     </row>
-    <row r="330" spans="1:18">
+    <row r="330" spans="1:18" hidden="1">
       <c r="A330" s="2" t="s">
         <v>570</v>
       </c>
@@ -30505,7 +30506,7 @@
         <v>63.322368421052637</v>
       </c>
     </row>
-    <row r="333" spans="1:18">
+    <row r="333" spans="1:18" hidden="1">
       <c r="A333" s="2" t="s">
         <v>573</v>
       </c>
@@ -30676,7 +30677,7 @@
         <v>84.046052631578945</v>
       </c>
     </row>
-    <row r="336" spans="1:18">
+    <row r="336" spans="1:18" hidden="1">
       <c r="A336" s="2" t="s">
         <v>576</v>
       </c>
@@ -30847,7 +30848,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="339" spans="1:18">
+    <row r="339" spans="1:18" hidden="1">
       <c r="A339" s="2" t="s">
         <v>579</v>
       </c>
@@ -31018,7 +31019,7 @@
         <v>60.394736842105267</v>
       </c>
     </row>
-    <row r="342" spans="1:18">
+    <row r="342" spans="1:18" hidden="1">
       <c r="A342" s="2" t="s">
         <v>582</v>
       </c>
@@ -31189,7 +31190,7 @@
         <v>139.4</v>
       </c>
     </row>
-    <row r="345" spans="1:18">
+    <row r="345" spans="1:18" hidden="1">
       <c r="A345" s="2" t="s">
         <v>585</v>
       </c>
@@ -31360,7 +31361,7 @@
         <v>63.35526315789474</v>
       </c>
     </row>
-    <row r="348" spans="1:18">
+    <row r="348" spans="1:18" hidden="1">
       <c r="A348" s="2" t="s">
         <v>588</v>
       </c>
@@ -31531,7 +31532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="351" spans="1:18">
+    <row r="351" spans="1:18" hidden="1">
       <c r="A351" s="2" t="s">
         <v>591</v>
       </c>
@@ -31702,7 +31703,7 @@
         <v>87.598684210526315</v>
       </c>
     </row>
-    <row r="354" spans="1:18">
+    <row r="354" spans="1:18" hidden="1">
       <c r="A354" s="2" t="s">
         <v>594</v>
       </c>
@@ -31873,7 +31874,7 @@
         <v>134.21052631578948</v>
       </c>
     </row>
-    <row r="357" spans="1:18">
+    <row r="357" spans="1:18" hidden="1">
       <c r="A357" s="2" t="s">
         <v>597</v>
       </c>
@@ -32044,7 +32045,7 @@
         <v>68.98026315789474</v>
       </c>
     </row>
-    <row r="360" spans="1:18">
+    <row r="360" spans="1:18" hidden="1">
       <c r="A360" s="2" t="s">
         <v>600</v>
       </c>
@@ -32215,7 +32216,7 @@
         <v>133.80000000000001</v>
       </c>
     </row>
-    <row r="363" spans="1:18">
+    <row r="363" spans="1:18" hidden="1">
       <c r="A363" s="2" t="s">
         <v>603</v>
       </c>
@@ -32386,7 +32387,7 @@
         <v>32.434210526315788</v>
       </c>
     </row>
-    <row r="366" spans="1:18">
+    <row r="366" spans="1:18" hidden="1">
       <c r="A366" s="2" t="s">
         <v>606</v>
       </c>
@@ -32557,7 +32558,7 @@
         <v>31.546052631578949</v>
       </c>
     </row>
-    <row r="369" spans="1:18">
+    <row r="369" spans="1:18" hidden="1">
       <c r="A369" s="2" t="s">
         <v>609</v>
       </c>
@@ -32728,7 +32729,7 @@
         <v>50.328947368421055</v>
       </c>
     </row>
-    <row r="372" spans="1:18">
+    <row r="372" spans="1:18" hidden="1">
       <c r="A372" s="2" t="s">
         <v>612</v>
       </c>
@@ -32899,7 +32900,7 @@
         <v>63.1</v>
       </c>
     </row>
-    <row r="375" spans="1:18">
+    <row r="375" spans="1:18" hidden="1">
       <c r="A375" s="2" t="s">
         <v>615</v>
       </c>
@@ -33070,7 +33071,7 @@
         <v>105.95394736842105</v>
       </c>
     </row>
-    <row r="378" spans="1:18">
+    <row r="378" spans="1:18" hidden="1">
       <c r="A378" s="2" t="s">
         <v>618</v>
       </c>
@@ -33241,7 +33242,7 @@
         <v>61.019736842105267</v>
       </c>
     </row>
-    <row r="381" spans="1:18">
+    <row r="381" spans="1:18" hidden="1">
       <c r="A381" s="2" t="s">
         <v>621</v>
       </c>
@@ -33412,7 +33413,7 @@
         <v>38.486842105263158</v>
       </c>
     </row>
-    <row r="384" spans="1:18">
+    <row r="384" spans="1:18" hidden="1">
       <c r="A384" s="2" t="s">
         <v>624</v>
       </c>
@@ -33583,7 +33584,7 @@
         <v>80.789473684210535</v>
       </c>
     </row>
-    <row r="387" spans="1:18">
+    <row r="387" spans="1:18" hidden="1">
       <c r="A387" s="2" t="s">
         <v>627</v>
       </c>
@@ -33754,7 +33755,7 @@
         <v>50.65789473684211</v>
       </c>
     </row>
-    <row r="390" spans="1:18">
+    <row r="390" spans="1:18" hidden="1">
       <c r="A390" s="2" t="s">
         <v>630</v>
       </c>
@@ -33925,7 +33926,7 @@
         <v>117.69736842105263</v>
       </c>
     </row>
-    <row r="393" spans="1:18">
+    <row r="393" spans="1:18" hidden="1">
       <c r="A393" s="2" t="s">
         <v>633</v>
       </c>
@@ -34096,7 +34097,7 @@
         <v>64.83552631578948</v>
       </c>
     </row>
-    <row r="396" spans="1:18">
+    <row r="396" spans="1:18" hidden="1">
       <c r="A396" s="2" t="s">
         <v>636</v>
       </c>
@@ -34267,7 +34268,7 @@
         <v>30.42763157894737</v>
       </c>
     </row>
-    <row r="399" spans="1:18">
+    <row r="399" spans="1:18" hidden="1">
       <c r="A399" s="2" t="s">
         <v>639</v>
       </c>
@@ -34438,7 +34439,7 @@
         <v>74.21052631578948</v>
       </c>
     </row>
-    <row r="402" spans="1:18">
+    <row r="402" spans="1:18" hidden="1">
       <c r="A402" s="2" t="s">
         <v>642</v>
       </c>
@@ -34609,7 +34610,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="405" spans="1:18">
+    <row r="405" spans="1:18" hidden="1">
       <c r="A405" s="2" t="s">
         <v>645</v>
       </c>
@@ -34780,7 +34781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="408" spans="1:18">
+    <row r="408" spans="1:18" hidden="1">
       <c r="A408" s="2" t="s">
         <v>648</v>
       </c>
@@ -34951,7 +34952,7 @@
         <v>62.894736842105267</v>
       </c>
     </row>
-    <row r="411" spans="1:18">
+    <row r="411" spans="1:18" hidden="1">
       <c r="A411" s="2" t="s">
         <v>651</v>
       </c>
@@ -35122,7 +35123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="414" spans="1:18">
+    <row r="414" spans="1:18" hidden="1">
       <c r="A414" s="2" t="s">
         <v>654</v>
       </c>
@@ -35293,7 +35294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="417" spans="1:18">
+    <row r="417" spans="1:18" hidden="1">
       <c r="A417" s="2" t="s">
         <v>657</v>
       </c>
@@ -35464,7 +35465,7 @@
         <v>31.776315789473685</v>
       </c>
     </row>
-    <row r="420" spans="1:18">
+    <row r="420" spans="1:18" hidden="1">
       <c r="A420" s="2" t="s">
         <v>660</v>
       </c>
@@ -35635,7 +35636,7 @@
         <v>144.1</v>
       </c>
     </row>
-    <row r="423" spans="1:18">
+    <row r="423" spans="1:18" hidden="1">
       <c r="A423" s="2" t="s">
         <v>663</v>
       </c>
@@ -35806,7 +35807,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="426" spans="1:18">
+    <row r="426" spans="1:18" hidden="1">
       <c r="A426" s="2" t="s">
         <v>666</v>
       </c>
@@ -36034,7 +36035,7 @@
         <v>36.200000000000003</v>
       </c>
     </row>
-    <row r="430" spans="1:18">
+    <row r="430" spans="1:18" hidden="1">
       <c r="A430" s="2" t="s">
         <v>670</v>
       </c>
@@ -36205,7 +36206,7 @@
         <v>51.875</v>
       </c>
     </row>
-    <row r="433" spans="1:18">
+    <row r="433" spans="1:18" hidden="1">
       <c r="A433" s="2" t="s">
         <v>673</v>
       </c>
@@ -36376,7 +36377,7 @@
         <v>52.7</v>
       </c>
     </row>
-    <row r="436" spans="1:18">
+    <row r="436" spans="1:18" hidden="1">
       <c r="A436" s="2" t="s">
         <v>676</v>
       </c>
@@ -36547,7 +36548,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="439" spans="1:18">
+    <row r="439" spans="1:18" hidden="1">
       <c r="A439" s="2" t="s">
         <v>679</v>
       </c>
@@ -36718,7 +36719,7 @@
         <v>148.30000000000001</v>
       </c>
     </row>
-    <row r="442" spans="1:18">
+    <row r="442" spans="1:18" hidden="1">
       <c r="A442" s="2" t="s">
         <v>682</v>
       </c>
@@ -36889,7 +36890,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="445" spans="1:18">
+    <row r="445" spans="1:18" hidden="1">
       <c r="A445" s="2" t="s">
         <v>685</v>
       </c>
@@ -37060,7 +37061,7 @@
         <v>44.013157894736842</v>
       </c>
     </row>
-    <row r="448" spans="1:18">
+    <row r="448" spans="1:18" hidden="1">
       <c r="A448" s="2" t="s">
         <v>688</v>
       </c>
@@ -37231,7 +37232,7 @@
         <v>39.835526315789473</v>
       </c>
     </row>
-    <row r="451" spans="1:18">
+    <row r="451" spans="1:18" hidden="1">
       <c r="A451" s="2" t="s">
         <v>691</v>
       </c>
@@ -37402,7 +37403,7 @@
         <v>138.61842105263159</v>
       </c>
     </row>
-    <row r="454" spans="1:18">
+    <row r="454" spans="1:18" hidden="1">
       <c r="A454" s="2" t="s">
         <v>694</v>
       </c>
@@ -37573,7 +37574,7 @@
         <v>24.013157894736842</v>
       </c>
     </row>
-    <row r="457" spans="1:18">
+    <row r="457" spans="1:18" hidden="1">
       <c r="A457" s="2" t="s">
         <v>697</v>
       </c>
@@ -37744,7 +37745,7 @@
         <v>42.138157894736842</v>
       </c>
     </row>
-    <row r="460" spans="1:18">
+    <row r="460" spans="1:18" hidden="1">
       <c r="A460" s="2" t="s">
         <v>700</v>
       </c>
@@ -37915,7 +37916,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="463" spans="1:18">
+    <row r="463" spans="1:18" hidden="1">
       <c r="A463" s="2" t="s">
         <v>703</v>
       </c>
@@ -38086,7 +38087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="466" spans="1:18">
+    <row r="466" spans="1:18" hidden="1">
       <c r="A466" s="2" t="s">
         <v>706</v>
       </c>
@@ -38257,7 +38258,7 @@
         <v>48.15789473684211</v>
       </c>
     </row>
-    <row r="469" spans="1:18">
+    <row r="469" spans="1:18" hidden="1">
       <c r="A469" s="2" t="s">
         <v>709</v>
       </c>
@@ -38428,7 +38429,7 @@
         <v>64.868421052631575</v>
       </c>
     </row>
-    <row r="472" spans="1:18">
+    <row r="472" spans="1:18" hidden="1">
       <c r="A472" s="2" t="s">
         <v>712</v>
       </c>
@@ -38599,7 +38600,7 @@
         <v>49.309210526315795</v>
       </c>
     </row>
-    <row r="475" spans="1:18">
+    <row r="475" spans="1:18" hidden="1">
       <c r="A475" s="2" t="s">
         <v>715</v>
       </c>
@@ -38770,7 +38771,7 @@
         <v>27.7</v>
       </c>
     </row>
-    <row r="478" spans="1:18">
+    <row r="478" spans="1:18" hidden="1">
       <c r="A478" s="2" t="s">
         <v>718</v>
       </c>
@@ -38941,7 +38942,7 @@
         <v>85.69078947368422</v>
       </c>
     </row>
-    <row r="481" spans="1:18">
+    <row r="481" spans="1:18" hidden="1">
       <c r="A481" s="2" t="s">
         <v>721</v>
       </c>
@@ -39112,7 +39113,7 @@
         <v>86.64473684210526</v>
       </c>
     </row>
-    <row r="484" spans="1:18">
+    <row r="484" spans="1:18" hidden="1">
       <c r="A484" s="2" t="s">
         <v>724</v>
       </c>
@@ -39283,7 +39284,7 @@
         <v>99.703947368421055</v>
       </c>
     </row>
-    <row r="487" spans="1:18">
+    <row r="487" spans="1:18" hidden="1">
       <c r="A487" s="2" t="s">
         <v>727</v>
       </c>
@@ -39454,7 +39455,7 @@
         <v>61.7</v>
       </c>
     </row>
-    <row r="490" spans="1:18">
+    <row r="490" spans="1:18" hidden="1">
       <c r="A490" s="2" t="s">
         <v>730</v>
       </c>
@@ -39625,7 +39626,7 @@
         <v>35.700000000000003</v>
       </c>
     </row>
-    <row r="493" spans="1:18">
+    <row r="493" spans="1:18" hidden="1">
       <c r="A493" s="2" t="s">
         <v>733</v>
       </c>
@@ -39796,7 +39797,7 @@
         <v>104.17763157894737</v>
       </c>
     </row>
-    <row r="496" spans="1:18">
+    <row r="496" spans="1:18" hidden="1">
       <c r="A496" s="2" t="s">
         <v>736</v>
       </c>
@@ -39967,7 +39968,7 @@
         <v>103.05921052631579</v>
       </c>
     </row>
-    <row r="499" spans="1:18">
+    <row r="499" spans="1:18" hidden="1">
       <c r="A499" s="2" t="s">
         <v>739</v>
       </c>
@@ -40138,7 +40139,7 @@
         <v>9.9</v>
       </c>
     </row>
-    <row r="502" spans="1:18">
+    <row r="502" spans="1:18" hidden="1">
       <c r="A502" s="2" t="s">
         <v>742</v>
       </c>
@@ -40309,7 +40310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="505" spans="1:18">
+    <row r="505" spans="1:18" hidden="1">
       <c r="A505" s="2" t="s">
         <v>745</v>
       </c>
@@ -40480,7 +40481,7 @@
         <v>101.61184210526316</v>
       </c>
     </row>
-    <row r="508" spans="1:18">
+    <row r="508" spans="1:18" hidden="1">
       <c r="A508" s="2" t="s">
         <v>748</v>
       </c>
@@ -40651,7 +40652,7 @@
         <v>21.973684210526315</v>
       </c>
     </row>
-    <row r="511" spans="1:18">
+    <row r="511" spans="1:18" hidden="1">
       <c r="A511" s="2" t="s">
         <v>751</v>
       </c>
@@ -40822,7 +40823,7 @@
         <v>55.1</v>
       </c>
     </row>
-    <row r="514" spans="1:18">
+    <row r="514" spans="1:18" hidden="1">
       <c r="A514" s="2" t="s">
         <v>754</v>
       </c>
@@ -40993,7 +40994,7 @@
         <v>59.901315789473685</v>
       </c>
     </row>
-    <row r="517" spans="1:18">
+    <row r="517" spans="1:18" hidden="1">
       <c r="A517" s="2" t="s">
         <v>757</v>
       </c>
@@ -41164,7 +41165,7 @@
         <v>77.10526315789474</v>
       </c>
     </row>
-    <row r="520" spans="1:18">
+    <row r="520" spans="1:18" hidden="1">
       <c r="A520" s="2" t="s">
         <v>760</v>
       </c>
@@ -41335,7 +41336,7 @@
         <v>40.299999999999997</v>
       </c>
     </row>
-    <row r="523" spans="1:18">
+    <row r="523" spans="1:18" hidden="1">
       <c r="A523" s="2" t="s">
         <v>763</v>
       </c>
@@ -41506,7 +41507,7 @@
         <v>11.3</v>
       </c>
     </row>
-    <row r="526" spans="1:18">
+    <row r="526" spans="1:18" hidden="1">
       <c r="A526" s="2" t="s">
         <v>766</v>
       </c>
@@ -41677,7 +41678,7 @@
         <v>62.92763157894737</v>
       </c>
     </row>
-    <row r="529" spans="1:18">
+    <row r="529" spans="1:18" hidden="1">
       <c r="A529" s="2" t="s">
         <v>769</v>
       </c>
@@ -41848,7 +41849,7 @@
         <v>77.73026315789474</v>
       </c>
     </row>
-    <row r="532" spans="1:18">
+    <row r="532" spans="1:18" hidden="1">
       <c r="A532" s="2" t="s">
         <v>772</v>
       </c>
@@ -42019,7 +42020,7 @@
         <v>79.309210526315795</v>
       </c>
     </row>
-    <row r="535" spans="1:18">
+    <row r="535" spans="1:18" hidden="1">
       <c r="A535" s="2" t="s">
         <v>775</v>
       </c>
@@ -42190,7 +42191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="538" spans="1:18">
+    <row r="538" spans="1:18" hidden="1">
       <c r="A538" s="2" t="s">
         <v>778</v>
       </c>
@@ -42361,7 +42362,7 @@
         <v>60.296052631578952</v>
       </c>
     </row>
-    <row r="541" spans="1:18">
+    <row r="541" spans="1:18" hidden="1">
       <c r="A541" s="2" t="s">
         <v>781</v>
       </c>
@@ -42532,7 +42533,7 @@
         <v>68.35526315789474</v>
       </c>
     </row>
-    <row r="544" spans="1:18">
+    <row r="544" spans="1:18" hidden="1">
       <c r="A544" s="2" t="s">
         <v>784</v>
       </c>
@@ -42703,7 +42704,7 @@
         <v>72.401315789473685</v>
       </c>
     </row>
-    <row r="547" spans="1:18">
+    <row r="547" spans="1:18" hidden="1">
       <c r="A547" s="2" t="s">
         <v>787</v>
       </c>
@@ -42874,7 +42875,7 @@
         <v>57.7</v>
       </c>
     </row>
-    <row r="550" spans="1:18">
+    <row r="550" spans="1:18" hidden="1">
       <c r="A550" s="2" t="s">
         <v>790</v>
       </c>
@@ -43045,7 +43046,7 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="553" spans="1:18">
+    <row r="553" spans="1:18" hidden="1">
       <c r="A553" s="2" t="s">
         <v>793</v>
       </c>
@@ -43216,7 +43217,7 @@
         <v>38.125</v>
       </c>
     </row>
-    <row r="556" spans="1:18">
+    <row r="556" spans="1:18" hidden="1">
       <c r="A556" s="2" t="s">
         <v>796</v>
       </c>
@@ -43387,7 +43388,7 @@
         <v>66.28289473684211</v>
       </c>
     </row>
-    <row r="559" spans="1:18">
+    <row r="559" spans="1:18" hidden="1">
       <c r="A559" s="2" t="s">
         <v>799</v>
       </c>
@@ -43558,7 +43559,7 @@
         <v>56.414473684210527</v>
       </c>
     </row>
-    <row r="562" spans="1:18">
+    <row r="562" spans="1:18" hidden="1">
       <c r="A562" s="2" t="s">
         <v>802</v>
       </c>
@@ -43729,7 +43730,7 @@
         <v>63.881578947368425</v>
       </c>
     </row>
-    <row r="565" spans="1:18">
+    <row r="565" spans="1:18" hidden="1">
       <c r="A565" s="2" t="s">
         <v>805</v>
       </c>
@@ -43900,7 +43901,7 @@
         <v>60.822368421052637</v>
       </c>
     </row>
-    <row r="568" spans="1:18">
+    <row r="568" spans="1:18" hidden="1">
       <c r="A568" s="2" t="s">
         <v>808</v>
       </c>
@@ -44071,7 +44072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="571" spans="1:18">
+    <row r="571" spans="1:18" hidden="1">
       <c r="A571" s="2" t="s">
         <v>811</v>
       </c>
@@ -44242,7 +44243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="574" spans="1:18">
+    <row r="574" spans="1:18" hidden="1">
       <c r="A574" s="2" t="s">
         <v>814</v>
       </c>
@@ -44413,7 +44414,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="577" spans="1:18">
+    <row r="577" spans="1:18" hidden="1">
       <c r="A577" s="2" t="s">
         <v>817</v>
       </c>
@@ -44584,7 +44585,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="580" spans="1:18">
+    <row r="580" spans="1:18" hidden="1">
       <c r="A580" s="2" t="s">
         <v>820</v>
       </c>
@@ -44755,7 +44756,7 @@
         <v>61.08552631578948</v>
       </c>
     </row>
-    <row r="583" spans="1:18">
+    <row r="583" spans="1:18" hidden="1">
       <c r="A583" s="2" t="s">
         <v>823</v>
       </c>
@@ -44926,7 +44927,7 @@
         <v>60.098684210526322</v>
       </c>
     </row>
-    <row r="586" spans="1:18">
+    <row r="586" spans="1:18" hidden="1">
       <c r="A586" s="2" t="s">
         <v>826</v>
       </c>
@@ -45097,7 +45098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="589" spans="1:18">
+    <row r="589" spans="1:18" hidden="1">
       <c r="A589" s="2" t="s">
         <v>829</v>
       </c>
@@ -45268,7 +45269,7 @@
         <v>51.118421052631582</v>
       </c>
     </row>
-    <row r="592" spans="1:18">
+    <row r="592" spans="1:18" hidden="1">
       <c r="A592" s="2" t="s">
         <v>832</v>
       </c>
@@ -45439,7 +45440,7 @@
         <v>82.92763157894737</v>
       </c>
     </row>
-    <row r="595" spans="1:18">
+    <row r="595" spans="1:18" hidden="1">
       <c r="A595" s="2" t="s">
         <v>835</v>
       </c>
@@ -45610,7 +45611,7 @@
         <v>62.664473684210527</v>
       </c>
     </row>
-    <row r="598" spans="1:18">
+    <row r="598" spans="1:18" hidden="1">
       <c r="A598" s="15" t="s">
         <v>1349</v>
       </c>
@@ -45778,7 +45779,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="601" spans="1:18">
+    <row r="601" spans="1:18" hidden="1">
       <c r="A601" s="15" t="s">
         <v>1350</v>
       </c>
@@ -45834,7 +45835,7 @@
         <v>103.83333333333333</v>
       </c>
     </row>
-    <row r="602" spans="1:18" ht="17">
+    <row r="602" spans="1:18" ht="17" hidden="1">
       <c r="A602" s="15" t="s">
         <v>1351</v>
       </c>
@@ -46002,7 +46003,7 @@
         <v>101.16666666666667</v>
       </c>
     </row>
-    <row r="605" spans="1:18">
+    <row r="605" spans="1:18" hidden="1">
       <c r="A605" s="15" t="s">
         <v>1352</v>
       </c>
@@ -46058,7 +46059,7 @@
         <v>116.5</v>
       </c>
     </row>
-    <row r="606" spans="1:18">
+    <row r="606" spans="1:18" hidden="1">
       <c r="A606" s="15" t="s">
         <v>1353</v>
       </c>
@@ -46226,7 +46227,7 @@
         <v>9.5833333333333339</v>
       </c>
     </row>
-    <row r="609" spans="1:18">
+    <row r="609" spans="1:18" hidden="1">
       <c r="A609" s="15" t="s">
         <v>1354</v>
       </c>
@@ -46282,7 +46283,7 @@
         <v>9.0833333333333339</v>
       </c>
     </row>
-    <row r="610" spans="1:18">
+    <row r="610" spans="1:18" hidden="1">
       <c r="A610" s="15" t="s">
         <v>1355</v>
       </c>
@@ -46450,7 +46451,7 @@
         <v>4.833333333333333</v>
       </c>
     </row>
-    <row r="613" spans="1:18">
+    <row r="613" spans="1:18" hidden="1">
       <c r="A613" s="15" t="s">
         <v>1356</v>
       </c>
@@ -46618,7 +46619,7 @@
         <v>54.666666666666664</v>
       </c>
     </row>
-    <row r="616" spans="1:18">
+    <row r="616" spans="1:18" hidden="1">
       <c r="A616" s="15" t="s">
         <v>1357</v>
       </c>
@@ -46786,7 +46787,7 @@
         <v>18.916666666666668</v>
       </c>
     </row>
-    <row r="619" spans="1:18">
+    <row r="619" spans="1:18" hidden="1">
       <c r="A619" s="15" t="s">
         <v>1358</v>
       </c>
@@ -46842,7 +46843,7 @@
         <v>43.333333333333336</v>
       </c>
     </row>
-    <row r="620" spans="1:18">
+    <row r="620" spans="1:18" hidden="1">
       <c r="A620" s="15" t="s">
         <v>1359</v>
       </c>
@@ -47010,7 +47011,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="623" spans="1:18">
+    <row r="623" spans="1:18" hidden="1">
       <c r="A623" s="15" t="s">
         <v>1360</v>
       </c>
@@ -47178,7 +47179,7 @@
         <v>32.5</v>
       </c>
     </row>
-    <row r="626" spans="1:18">
+    <row r="626" spans="1:18" hidden="1">
       <c r="A626" s="15" t="s">
         <v>1361</v>
       </c>
@@ -47346,7 +47347,7 @@
         <v>47.833333333333336</v>
       </c>
     </row>
-    <row r="629" spans="1:18">
+    <row r="629" spans="1:18" hidden="1">
       <c r="A629" s="15" t="s">
         <v>1362</v>
       </c>
@@ -47514,7 +47515,7 @@
         <v>3.6666666666666665</v>
       </c>
     </row>
-    <row r="632" spans="1:18">
+    <row r="632" spans="1:18" hidden="1">
       <c r="A632" s="15" t="s">
         <v>1363</v>
       </c>
@@ -47682,7 +47683,7 @@
         <v>21.666666666666668</v>
       </c>
     </row>
-    <row r="635" spans="1:18">
+    <row r="635" spans="1:18" hidden="1">
       <c r="A635" s="15" t="s">
         <v>1364</v>
       </c>
@@ -47850,7 +47851,7 @@
         <v>9.5833333333333339</v>
       </c>
     </row>
-    <row r="638" spans="1:18" ht="17">
+    <row r="638" spans="1:18" ht="17" hidden="1">
       <c r="A638" s="15" t="s">
         <v>1365</v>
       </c>
@@ -48018,7 +48019,7 @@
         <v>17.666666666666668</v>
       </c>
     </row>
-    <row r="641" spans="1:18">
+    <row r="641" spans="1:18" hidden="1">
       <c r="A641" s="15" t="s">
         <v>1366</v>
       </c>
@@ -48186,7 +48187,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="644" spans="1:18">
+    <row r="644" spans="1:18" hidden="1">
       <c r="A644" s="15" t="s">
         <v>1367</v>
       </c>
@@ -48354,7 +48355,7 @@
         <v>5.583333333333333</v>
       </c>
     </row>
-    <row r="647" spans="1:18">
+    <row r="647" spans="1:18" hidden="1">
       <c r="A647" s="15" t="s">
         <v>1368</v>
       </c>
@@ -48522,7 +48523,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="650" spans="1:18">
+    <row r="650" spans="1:18" hidden="1">
       <c r="A650" s="15" t="s">
         <v>1369</v>
       </c>
@@ -48690,7 +48691,7 @@
         <v>32.416666666666664</v>
       </c>
     </row>
-    <row r="653" spans="1:18">
+    <row r="653" spans="1:18" hidden="1">
       <c r="A653" s="15" t="s">
         <v>1370</v>
       </c>
@@ -48858,7 +48859,7 @@
         <v>31.25</v>
       </c>
     </row>
-    <row r="656" spans="1:18">
+    <row r="656" spans="1:18" hidden="1">
       <c r="A656" s="15" t="s">
         <v>1371</v>
       </c>
@@ -49026,7 +49027,7 @@
         <v>4.583333333333333</v>
       </c>
     </row>
-    <row r="659" spans="1:18">
+    <row r="659" spans="1:18" hidden="1">
       <c r="A659" s="15" t="s">
         <v>1372</v>
       </c>
@@ -49194,7 +49195,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="662" spans="1:18">
+    <row r="662" spans="1:18" hidden="1">
       <c r="A662" s="15" t="s">
         <v>1373</v>
       </c>
@@ -49362,7 +49363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="665" spans="1:18">
+    <row r="665" spans="1:18" hidden="1">
       <c r="A665" s="15" t="s">
         <v>1374</v>
       </c>
@@ -49530,7 +49531,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="668" spans="1:18">
+    <row r="668" spans="1:18" hidden="1">
       <c r="A668" s="15" t="s">
         <v>1375</v>
       </c>
@@ -49698,7 +49699,7 @@
         <v>49.166666666666664</v>
       </c>
     </row>
-    <row r="671" spans="1:18" ht="17">
+    <row r="671" spans="1:18" ht="17" hidden="1">
       <c r="A671" s="15" t="s">
         <v>1376</v>
       </c>
@@ -49866,7 +49867,7 @@
         <v>4.416666666666667</v>
       </c>
     </row>
-    <row r="674" spans="1:18">
+    <row r="674" spans="1:18" hidden="1">
       <c r="A674" s="15" t="s">
         <v>1377</v>
       </c>
@@ -50034,7 +50035,7 @@
         <v>4.416666666666667</v>
       </c>
     </row>
-    <row r="677" spans="1:18">
+    <row r="677" spans="1:18" hidden="1">
       <c r="A677" s="15" t="s">
         <v>1378</v>
       </c>
@@ -50202,7 +50203,7 @@
         <v>5.583333333333333</v>
       </c>
     </row>
-    <row r="680" spans="1:18">
+    <row r="680" spans="1:18" hidden="1">
       <c r="A680" s="15" t="s">
         <v>1379</v>
       </c>
@@ -50370,7 +50371,7 @@
         <v>35.75</v>
       </c>
     </row>
-    <row r="683" spans="1:18">
+    <row r="683" spans="1:18" hidden="1">
       <c r="A683" s="15" t="s">
         <v>1380</v>
       </c>
@@ -50538,7 +50539,7 @@
         <v>9.25</v>
       </c>
     </row>
-    <row r="686" spans="1:18">
+    <row r="686" spans="1:18" hidden="1">
       <c r="A686" s="15" t="s">
         <v>1381</v>
       </c>
@@ -50706,7 +50707,7 @@
         <v>74.25</v>
       </c>
     </row>
-    <row r="689" spans="1:18">
+    <row r="689" spans="1:18" hidden="1">
       <c r="A689" s="15" t="s">
         <v>1382</v>
       </c>
@@ -50874,7 +50875,7 @@
         <v>47.833333333333336</v>
       </c>
     </row>
-    <row r="692" spans="1:18">
+    <row r="692" spans="1:18" hidden="1">
       <c r="A692" s="15" t="s">
         <v>1383</v>
       </c>
@@ -51042,7 +51043,7 @@
         <v>3.25</v>
       </c>
     </row>
-    <row r="695" spans="1:18">
+    <row r="695" spans="1:18" hidden="1">
       <c r="A695" s="15" t="s">
         <v>1384</v>
       </c>
@@ -51210,7 +51211,7 @@
         <v>12.5</v>
       </c>
     </row>
-    <row r="698" spans="1:18">
+    <row r="698" spans="1:18" hidden="1">
       <c r="A698" s="15" t="s">
         <v>1385</v>
       </c>
@@ -51378,7 +51379,7 @@
         <v>18.75</v>
       </c>
     </row>
-    <row r="701" spans="1:18">
+    <row r="701" spans="1:18" hidden="1">
       <c r="A701" s="15" t="s">
         <v>1386</v>
       </c>
@@ -51546,7 +51547,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="704" spans="1:18">
+    <row r="704" spans="1:18" hidden="1">
       <c r="A704" s="15" t="s">
         <v>1387</v>
       </c>
@@ -51714,7 +51715,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="707" spans="1:18">
+    <row r="707" spans="1:18" hidden="1">
       <c r="A707" s="15" t="s">
         <v>1388</v>
       </c>
@@ -51893,12 +51894,20 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:R709" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="FFPE block"/>
+        <filter val="OCT Block"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A598:R709">
     <sortCondition ref="B598:B709"/>
     <sortCondition ref="D598:D709"/>
   </sortState>
   <phoneticPr fontId="4" type="noConversion"/>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="custom" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="length &lt;15 characters, no space or symbols allowed expect underscore &quot;_&quot;" prompt="length &lt;15 characters, no space or symbols allowed expect underscore &quot;_&quot;" sqref="A56:A225 B2:B55 C2:C227" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>AND(ISTEXT(A2),LEN(A2)&lt;16,ISERROR(FIND("-",A2)),ISERROR(FIND("+",A2)),ISERROR(FIND(" ",A2)))</formula1>
     </dataValidation>
@@ -51918,6 +51927,24 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="856faa8c-3633-4dde-8999-5e4660e8562b" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="44ef09d3-2911-4fbe-94dd-fad613be0447">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Firstauthor xmlns="44ef09d3-2911-4fbe-94dd-fad613be0447" xsi:nil="true"/>
+    <YourName xmlns="44ef09d3-2911-4fbe-94dd-fad613be0447" xsi:nil="true"/>
+    <BriefSummary xmlns="44ef09d3-2911-4fbe-94dd-fad613be0447" xsi:nil="true"/>
+    <Journalname xmlns="44ef09d3-2911-4fbe-94dd-fad613be0447" xsi:nil="true"/>
+    <Date xmlns="44ef09d3-2911-4fbe-94dd-fad613be0447" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100969C1FEA7402A04796BFBD957B7C1FFF" ma:contentTypeVersion="26" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cc2fb7094e8a4f3be50808662b69bbb1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="856faa8c-3633-4dde-8999-5e4660e8562b" xmlns:ns3="44ef09d3-2911-4fbe-94dd-fad613be0447" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1e3a05a934d72aef0c07279d5f4f5d6f" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -52231,24 +52258,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="856faa8c-3633-4dde-8999-5e4660e8562b" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="44ef09d3-2911-4fbe-94dd-fad613be0447">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Firstauthor xmlns="44ef09d3-2911-4fbe-94dd-fad613be0447" xsi:nil="true"/>
-    <YourName xmlns="44ef09d3-2911-4fbe-94dd-fad613be0447" xsi:nil="true"/>
-    <BriefSummary xmlns="44ef09d3-2911-4fbe-94dd-fad613be0447" xsi:nil="true"/>
-    <Journalname xmlns="44ef09d3-2911-4fbe-94dd-fad613be0447" xsi:nil="true"/>
-    <Date xmlns="44ef09d3-2911-4fbe-94dd-fad613be0447" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03E62BC1-1663-47D5-ACC5-74C03EAE98F0}">
   <ds:schemaRefs>
@@ -52258,6 +52267,24 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{35795E13-7B99-4083-B536-CC6B4C6F1652}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="44ef09d3-2911-4fbe-94dd-fad613be0447"/>
+    <ds:schemaRef ds:uri="856faa8c-3633-4dde-8999-5e4660e8562b"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{135595A6-845F-4594-9B73-C4998094A7C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -52277,26 +52304,9 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{35795E13-7B99-4083-B536-CC6B4C6F1652}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="856faa8c-3633-4dde-8999-5e4660e8562b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="44ef09d3-2911-4fbe-94dd-fad613be0447"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{14b77578-9773-42d5-8507-251ca2dc2b06}" enabled="0" method="" siteId="{14b77578-9773-42d5-8507-251ca2dc2b06}" removed="1"/>
+  <clbl:label id="{717009a6-20de-461a-8894-0312a395cac9}" enabled="0" method="" siteId="{717009a6-20de-461a-8894-0312a395cac9}" removed="1"/>
 </clbl:labelList>
 </file>
</xml_diff>